<commit_message>
[auto-snapshot] 2026-04-28 12:00 | onda-hompage | 34 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_nail/광주_네일샵.xlsx
+++ b/naver-place-crawler/results_nail/광주_네일샵.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -564,29 +564,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>네일더빛나 페디크루 광주전대점 내성발톱 무좀 발각질</t>
+          <t>네일홀릭 학동본점</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>jisu1980@naver.com</t>
+          <t>nailholicshop@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1399-3236</t>
+          <t>0507-1334-0423</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>광주 북구 서방로9번길 12 2층 네일더빛나 전대점</t>
+          <t>광주 동구 학소로 125 105호</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/jisu1980</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -596,24 +596,20 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4dwzd</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>X</t>
@@ -625,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>1167</v>
+        <v>83</v>
       </c>
       <c r="Q2" t="n">
-        <v>952</v>
+        <v>8</v>
       </c>
       <c r="R2" t="n">
-        <v>2119</v>
+        <v>91</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -640,17 +636,17 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1824211380</t>
+          <t>34079967</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1824211380</t>
+          <t>https://m.place.naver.com/place/34079967</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -662,29 +658,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>네일홀릭 학동본점</t>
+          <t>네일플롯 광주첨단점</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>nailholicshop@naver.com</t>
+          <t>nailflot@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1334-0423</t>
+          <t>0507-1377-2701</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>광주 동구 학소로 125 105호</t>
+          <t>광주 광산구 임방울대로826번길 47 2층 201호 네일플롯</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/nailholicshop</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -694,23 +690,27 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>https://talk.naver.com/ct/w47h6j</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -719,13 +719,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>83</v>
+        <v>2112</v>
       </c>
       <c r="Q3" t="n">
-        <v>8</v>
+        <v>177</v>
       </c>
       <c r="R3" t="n">
-        <v>91</v>
+        <v>2289</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -734,17 +734,17 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>34079967</t>
+          <t>1760350557</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/34079967</t>
+          <t>https://m.place.naver.com/place/1760350557</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -756,29 +756,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>네일플롯 광주첨단점</t>
+          <t>네일더빛나 페디크루 광주전대점 내성발톱 무좀 발각질</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>nailflot@naver.com</t>
+          <t>jisu1980@naver.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1377-2701</t>
+          <t>0507-1399-3236</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>광주 광산구 임방울대로826번길 47 2층 201호 네일플롯</t>
+          <t>광주 북구 서방로9번길 12 2층 네일더빛나 전대점</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>http://www.instagram.com/flot_nail</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -803,12 +803,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://talk.naver.com/ct/w47h6j</t>
+          <t>https://talk.naver.com/ct/w4dwzd</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -817,13 +817,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>2111</v>
+        <v>1167</v>
       </c>
       <c r="Q4" t="n">
-        <v>177</v>
+        <v>953</v>
       </c>
       <c r="R4" t="n">
-        <v>2288</v>
+        <v>2120</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -832,17 +832,17 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1760350557</t>
+          <t>1824211380</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1760350557</t>
+          <t>https://m.place.naver.com/place/1824211380</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/hosinail_</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1016,10 +1016,10 @@
         <v>1553</v>
       </c>
       <c r="Q6" t="n">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="R6" t="n">
-        <v>2350</v>
+        <v>2352</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1144,29 +1144,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>리보니 오로지푸스 무좀 내성발톱 발각질 맞춤깔창</t>
+          <t>우아한네일</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>rebornee__@naver.com</t>
+          <t>kqw1230@naver.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0507-1388-0801</t>
+          <t>0507-1472-3402</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>광주 남구 대남대로283번길 8 1층</t>
+          <t>광주 서구 상무화원로 12 1층 우아한네일</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/rebornee__</t>
+          <t>https://www.instagram.com/wooahan_nail</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1181,19 +1181,15 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w5w1hn</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>X</t>
@@ -1205,13 +1201,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>243</v>
+        <v>457</v>
       </c>
       <c r="Q8" t="n">
-        <v>45</v>
+        <v>211</v>
       </c>
       <c r="R8" t="n">
-        <v>288</v>
+        <v>668</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1220,17 +1216,17 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1375528945</t>
+          <t>1384925755</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1375528945</t>
+          <t>https://m.place.naver.com/place/1384925755</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1242,34 +1238,34 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>아임뷰티</t>
+          <t>리보니 오로지푸스 무좀 내성발톱 발각질 맞춤깔창</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>wldyd3412@naver.com</t>
+          <t>rebornee__@naver.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0507-1328-6485</t>
+          <t>0507-1388-0801</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>광주 광산구 앰코로 35 3층 312-1호</t>
+          <t>광주 남구 대남대로283번길 8 1층</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/im_beauty_nail_?igsh=cGY0b3Bhano0dzR5</t>
+          <t>https://blog.naver.com/rebornee__</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1289,7 +1285,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://talk.naver.com/ct/w49mnk</t>
+          <t>https://talk.naver.com/ct/w5w1hn</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1303,13 +1299,13 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>312</v>
+        <v>243</v>
       </c>
       <c r="Q9" t="n">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="R9" t="n">
-        <v>381</v>
+        <v>288</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1318,17 +1314,17 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1323398142</t>
+          <t>1375528945</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1323398142</t>
+          <t>https://m.place.naver.com/place/1375528945</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1418,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1516,101 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>원하다뷰티</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>moonda09120@naver.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>광주 광산구 산월로 17 1층 원하다뷰티</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://talk.naver.com/ct/w436o4</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>456</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>59</v>
+      </c>
+      <c r="R12" t="n">
+        <v>515</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>1007616332</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1007616332</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>

</xml_diff>